<commit_message>
fix decoding for gen_test_vectors script for netio
</commit_message>
<xml_diff>
--- a/gen_test_vectors/test_vectors.xlsx
+++ b/gen_test_vectors/test_vectors.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ubcca-my.sharepoint.com/personal/harristm_student_ubc_ca/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{83022187-D316-48DC-BDF8-10E1781715CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{83022187-D316-48DC-BDF8-10E1781715CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{780E2EBF-4CFC-4A79-87F4-083AE7E5D68E}"/>
   <bookViews>
-    <workbookView xWindow="-16395" yWindow="3435" windowWidth="20130" windowHeight="11580" xr2:uid="{ED369803-A866-4415-A5F6-8FB9FD74AFF7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{ED369803-A866-4415-A5F6-8FB9FD74AFF7}"/>
   </bookViews>
   <sheets>
     <sheet name="NetIO_Test" sheetId="1" r:id="rId1"/>
@@ -499,6 +499,9 @@
       <c r="A2" t="s">
         <v>8</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2">
         <v>1</v>
       </c>
@@ -512,13 +515,16 @@
         <v>10</v>
       </c>
       <c r="G2" s="1">
-        <v>20</v>
+        <v>280</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>11</v>
       </c>
+      <c r="B3">
+        <v>4</v>
+      </c>
       <c r="C3">
         <v>1</v>
       </c>
@@ -532,13 +538,16 @@
         <v>10</v>
       </c>
       <c r="G3" s="1">
-        <v>20</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
       <c r="C4">
         <v>2</v>
       </c>
@@ -552,13 +561,16 @@
         <v>10</v>
       </c>
       <c r="G4" s="1">
-        <v>30.2</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
       <c r="C5">
         <v>2</v>
       </c>
@@ -572,7 +584,7 @@
         <v>10</v>
       </c>
       <c r="G5" s="1">
-        <v>30.2</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added test vector for algo
</commit_message>
<xml_diff>
--- a/gen_test_vectors/test_vectors.xlsx
+++ b/gen_test_vectors/test_vectors.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ubcca-my.sharepoint.com/personal/harristm_student_ubc_ca/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\sofiyasp\capstone\elec491-hft-system\gen_test_vectors\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{83022187-D316-48DC-BDF8-10E1781715CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{780E2EBF-4CFC-4A79-87F4-083AE7E5D68E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D64BD873-739F-4845-84EF-8ED89FE1550B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{ED369803-A866-4415-A5F6-8FB9FD74AFF7}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{ED369803-A866-4415-A5F6-8FB9FD74AFF7}"/>
   </bookViews>
   <sheets>
     <sheet name="NetIO_Test" sheetId="1" r:id="rId1"/>
+    <sheet name="Algo_Test" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="61">
   <si>
     <t>Message Type</t>
   </si>
@@ -72,6 +73,153 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>F001: Warmup - No orders expected</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>F001: Full fill</t>
+  </si>
+  <si>
+    <t>F001: Second warmup order</t>
+  </si>
+  <si>
+    <t>F003/F004: MACD Up-Cross - BUY</t>
+  </si>
+  <si>
+    <t>F003/F004: Fill on up-cross</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>F003/F004: MACD Down-Cross - SELL</t>
+  </si>
+  <si>
+    <t>F003/F004: Fill on down-cross</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>F005: Wide Spread (600bp) - REJECT</t>
+  </si>
+  <si>
+    <t>F006: Crossed Market (Bid &gt; Ask) - REJECT</t>
+  </si>
+  <si>
+    <t>F007: Order Reject from Exchange</t>
+  </si>
+  <si>
+    <t>F007: Exchange sends REJECT</t>
+  </si>
+  <si>
+    <t>F008: Order 2</t>
+  </si>
+  <si>
+    <t>F008: Order 3</t>
+  </si>
+  <si>
+    <t>F008: Order 4</t>
+  </si>
+  <si>
+    <t>F008: Order 5</t>
+  </si>
+  <si>
+    <t>F008: Order 6</t>
+  </si>
+  <si>
+    <t>F008: Order 7</t>
+  </si>
+  <si>
+    <t>F008: Order 8</t>
+  </si>
+  <si>
+    <t>F008: Order 9</t>
+  </si>
+  <si>
+    <t>F008: Order 10</t>
+  </si>
+  <si>
+    <t>F008: Order 11</t>
+  </si>
+  <si>
+    <t>F008: Order 12</t>
+  </si>
+  <si>
+    <t>F008: Order 13</t>
+  </si>
+  <si>
+    <t>F008: Order 14</t>
+  </si>
+  <si>
+    <t>F008: Order 15</t>
+  </si>
+  <si>
+    <t>F008: Drain order 2</t>
+  </si>
+  <si>
+    <t>F008: Drain order 3</t>
+  </si>
+  <si>
+    <t>F008: Drain order 4</t>
+  </si>
+  <si>
+    <t>F008: Drain order 5</t>
+  </si>
+  <si>
+    <t>F008: Drain order 6</t>
+  </si>
+  <si>
+    <t>F008: Drain order 7</t>
+  </si>
+  <si>
+    <t>F008: Drain order 8</t>
+  </si>
+  <si>
+    <t>F008: Drain order 9</t>
+  </si>
+  <si>
+    <t>F008: Drain order 10</t>
+  </si>
+  <si>
+    <t>F008: Drain order 11</t>
+  </si>
+  <si>
+    <t>F008: Drain order 12</t>
+  </si>
+  <si>
+    <t>F008: Drain order 13</t>
+  </si>
+  <si>
+    <t>F008: Drain order 14</t>
+  </si>
+  <si>
+    <t>F008: Drain order 15</t>
+  </si>
+  <si>
+    <t>F008: Drain order 16</t>
+  </si>
+  <si>
+    <t>F009: Partial Fill Test - BUY</t>
+  </si>
+  <si>
+    <t>F008: Backpressure Test</t>
+  </si>
+  <si>
+    <t>F008: Order 16 (MAX_OUT)</t>
+  </si>
+  <si>
+    <t>F008: Begin draining backlog</t>
+  </si>
+  <si>
+    <t>F009: Partial fill (50/100)</t>
+  </si>
+  <si>
+    <t>F009: Cancel remaining 50</t>
   </si>
 </sst>
 </file>
@@ -457,19 +605,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DF5265A-848D-41CC-91AC-C85D5FCC76DE}">
   <dimension ref="A1:H5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" customWidth="1"/>
-    <col min="3" max="3" width="10.140625" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" customWidth="1"/>
+    <col min="1" max="1" width="13.5546875" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" customWidth="1"/>
+    <col min="4" max="4" width="8.5546875" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" customWidth="1"/>
+    <col min="6" max="6" width="9.5546875" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" customWidth="1"/>
+    <col min="8" max="8" width="10.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -495,7 +643,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -518,7 +666,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -541,7 +689,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -564,7 +712,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -585,6 +733,1269 @@
       </c>
       <c r="G5" s="1">
         <v>281</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D6321DC-D19B-46D7-B7B5-9FA12476A606}">
+  <dimension ref="A1:H54"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.33203125" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="8" max="8" width="38.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1000</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2">
+        <v>100</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>299.91000000000003</v>
+      </c>
+      <c r="H2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>1000</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3">
+        <v>100</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3">
+        <v>299.91000000000003</v>
+      </c>
+      <c r="H3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>1001</v>
+      </c>
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4">
+        <v>100</v>
+      </c>
+      <c r="F4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4">
+        <v>299.91000000000003</v>
+      </c>
+      <c r="H4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>1001</v>
+      </c>
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5">
+        <v>100</v>
+      </c>
+      <c r="F5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5">
+        <v>299.91000000000003</v>
+      </c>
+      <c r="H5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7">
+        <v>1002</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7">
+        <v>100</v>
+      </c>
+      <c r="F7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7">
+        <v>309.91000000000003</v>
+      </c>
+      <c r="H7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8">
+        <v>1002</v>
+      </c>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8">
+        <v>100</v>
+      </c>
+      <c r="F8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8">
+        <v>309.91000000000003</v>
+      </c>
+      <c r="H8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>1003</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9">
+        <v>100</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9">
+        <v>289.91000000000003</v>
+      </c>
+      <c r="H9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="C10">
+        <v>1003</v>
+      </c>
+      <c r="D10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10">
+        <v>100</v>
+      </c>
+      <c r="F10" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10">
+        <v>289.91000000000003</v>
+      </c>
+      <c r="H10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12">
+        <v>9</v>
+      </c>
+      <c r="C12">
+        <v>1004</v>
+      </c>
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12">
+        <v>100</v>
+      </c>
+      <c r="F12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12">
+        <v>309.91000000000003</v>
+      </c>
+      <c r="H12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14">
+        <v>10</v>
+      </c>
+      <c r="C14">
+        <v>1005</v>
+      </c>
+      <c r="D14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14">
+        <v>100</v>
+      </c>
+      <c r="F14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14">
+        <v>309.91000000000003</v>
+      </c>
+      <c r="H14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16">
+        <v>11</v>
+      </c>
+      <c r="C16">
+        <v>1006</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16">
+        <v>100</v>
+      </c>
+      <c r="F16" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16">
+        <v>309.91000000000003</v>
+      </c>
+      <c r="H16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17">
+        <v>12</v>
+      </c>
+      <c r="C17">
+        <v>1006</v>
+      </c>
+      <c r="D17" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17">
+        <v>100</v>
+      </c>
+      <c r="F17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17">
+        <v>309.91000000000003</v>
+      </c>
+      <c r="H17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>8</v>
+      </c>
+      <c r="B19">
+        <v>13</v>
+      </c>
+      <c r="C19">
+        <v>1007</v>
+      </c>
+      <c r="D19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19">
+        <v>100</v>
+      </c>
+      <c r="F19" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19">
+        <v>309.91000000000003</v>
+      </c>
+      <c r="H19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20">
+        <v>14</v>
+      </c>
+      <c r="C20">
+        <v>1008</v>
+      </c>
+      <c r="D20" t="s">
+        <v>9</v>
+      </c>
+      <c r="E20">
+        <v>100</v>
+      </c>
+      <c r="F20" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20">
+        <v>310.41000000000003</v>
+      </c>
+      <c r="H20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B21">
+        <v>15</v>
+      </c>
+      <c r="C21">
+        <v>1009</v>
+      </c>
+      <c r="D21" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21">
+        <v>100</v>
+      </c>
+      <c r="F21" t="s">
+        <v>10</v>
+      </c>
+      <c r="G21">
+        <v>310.91000000000003</v>
+      </c>
+      <c r="H21" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22">
+        <v>16</v>
+      </c>
+      <c r="C22">
+        <v>1010</v>
+      </c>
+      <c r="D22" t="s">
+        <v>9</v>
+      </c>
+      <c r="E22">
+        <v>100</v>
+      </c>
+      <c r="F22" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22">
+        <v>311.41000000000003</v>
+      </c>
+      <c r="H22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23">
+        <v>17</v>
+      </c>
+      <c r="C23">
+        <v>1011</v>
+      </c>
+      <c r="D23" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23">
+        <v>100</v>
+      </c>
+      <c r="F23" t="s">
+        <v>10</v>
+      </c>
+      <c r="G23">
+        <v>311.91000000000003</v>
+      </c>
+      <c r="H23" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24">
+        <v>18</v>
+      </c>
+      <c r="C24">
+        <v>1012</v>
+      </c>
+      <c r="D24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E24">
+        <v>100</v>
+      </c>
+      <c r="F24" t="s">
+        <v>10</v>
+      </c>
+      <c r="G24">
+        <v>312.41000000000003</v>
+      </c>
+      <c r="H24" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>8</v>
+      </c>
+      <c r="B25">
+        <v>19</v>
+      </c>
+      <c r="C25">
+        <v>1013</v>
+      </c>
+      <c r="D25" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25">
+        <v>100</v>
+      </c>
+      <c r="F25" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25">
+        <v>312.91000000000003</v>
+      </c>
+      <c r="H25" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26">
+        <v>20</v>
+      </c>
+      <c r="C26">
+        <v>1014</v>
+      </c>
+      <c r="D26" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26">
+        <v>100</v>
+      </c>
+      <c r="F26" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26">
+        <v>313.41000000000003</v>
+      </c>
+      <c r="H26" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>8</v>
+      </c>
+      <c r="B27">
+        <v>21</v>
+      </c>
+      <c r="C27">
+        <v>1015</v>
+      </c>
+      <c r="D27" t="s">
+        <v>9</v>
+      </c>
+      <c r="E27">
+        <v>100</v>
+      </c>
+      <c r="F27" t="s">
+        <v>10</v>
+      </c>
+      <c r="G27">
+        <v>313.91000000000003</v>
+      </c>
+      <c r="H27" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28">
+        <v>22</v>
+      </c>
+      <c r="C28">
+        <v>1016</v>
+      </c>
+      <c r="D28" t="s">
+        <v>9</v>
+      </c>
+      <c r="E28">
+        <v>100</v>
+      </c>
+      <c r="F28" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28">
+        <v>314.41000000000003</v>
+      </c>
+      <c r="H28" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>8</v>
+      </c>
+      <c r="B29">
+        <v>23</v>
+      </c>
+      <c r="C29">
+        <v>1017</v>
+      </c>
+      <c r="D29" t="s">
+        <v>9</v>
+      </c>
+      <c r="E29">
+        <v>100</v>
+      </c>
+      <c r="F29" t="s">
+        <v>10</v>
+      </c>
+      <c r="G29">
+        <v>314.91000000000003</v>
+      </c>
+      <c r="H29" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30">
+        <v>24</v>
+      </c>
+      <c r="C30">
+        <v>1018</v>
+      </c>
+      <c r="D30" t="s">
+        <v>9</v>
+      </c>
+      <c r="E30">
+        <v>100</v>
+      </c>
+      <c r="F30" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30">
+        <v>315.41000000000003</v>
+      </c>
+      <c r="H30" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31">
+        <v>25</v>
+      </c>
+      <c r="C31">
+        <v>1019</v>
+      </c>
+      <c r="D31" t="s">
+        <v>9</v>
+      </c>
+      <c r="E31">
+        <v>100</v>
+      </c>
+      <c r="F31" t="s">
+        <v>10</v>
+      </c>
+      <c r="G31">
+        <v>315.91000000000003</v>
+      </c>
+      <c r="H31" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>8</v>
+      </c>
+      <c r="B32">
+        <v>26</v>
+      </c>
+      <c r="C32">
+        <v>1020</v>
+      </c>
+      <c r="D32" t="s">
+        <v>9</v>
+      </c>
+      <c r="E32">
+        <v>100</v>
+      </c>
+      <c r="F32" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32">
+        <v>316.41000000000003</v>
+      </c>
+      <c r="H32" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33">
+        <v>27</v>
+      </c>
+      <c r="C33">
+        <v>1021</v>
+      </c>
+      <c r="D33" t="s">
+        <v>9</v>
+      </c>
+      <c r="E33">
+        <v>100</v>
+      </c>
+      <c r="F33" t="s">
+        <v>10</v>
+      </c>
+      <c r="G33">
+        <v>316.91000000000003</v>
+      </c>
+      <c r="H33" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>8</v>
+      </c>
+      <c r="B34">
+        <v>28</v>
+      </c>
+      <c r="C34">
+        <v>1022</v>
+      </c>
+      <c r="D34" t="s">
+        <v>9</v>
+      </c>
+      <c r="E34">
+        <v>100</v>
+      </c>
+      <c r="F34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34">
+        <v>317.41000000000003</v>
+      </c>
+      <c r="H34" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35">
+        <v>29</v>
+      </c>
+      <c r="C35">
+        <v>1007</v>
+      </c>
+      <c r="D35" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35">
+        <v>100</v>
+      </c>
+      <c r="F35" t="s">
+        <v>10</v>
+      </c>
+      <c r="G35">
+        <v>309.91000000000003</v>
+      </c>
+      <c r="H35" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>13</v>
+      </c>
+      <c r="B36">
+        <v>30</v>
+      </c>
+      <c r="C36">
+        <v>1008</v>
+      </c>
+      <c r="D36" t="s">
+        <v>9</v>
+      </c>
+      <c r="E36">
+        <v>100</v>
+      </c>
+      <c r="F36" t="s">
+        <v>10</v>
+      </c>
+      <c r="G36">
+        <v>310.41000000000003</v>
+      </c>
+      <c r="H36" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37">
+        <v>31</v>
+      </c>
+      <c r="C37">
+        <v>1009</v>
+      </c>
+      <c r="D37" t="s">
+        <v>9</v>
+      </c>
+      <c r="E37">
+        <v>100</v>
+      </c>
+      <c r="F37" t="s">
+        <v>10</v>
+      </c>
+      <c r="G37">
+        <v>310.91000000000003</v>
+      </c>
+      <c r="H37" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38">
+        <v>32</v>
+      </c>
+      <c r="C38">
+        <v>1010</v>
+      </c>
+      <c r="D38" t="s">
+        <v>9</v>
+      </c>
+      <c r="E38">
+        <v>100</v>
+      </c>
+      <c r="F38" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38">
+        <v>311.41000000000003</v>
+      </c>
+      <c r="H38" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>13</v>
+      </c>
+      <c r="B39">
+        <v>33</v>
+      </c>
+      <c r="C39">
+        <v>1011</v>
+      </c>
+      <c r="D39" t="s">
+        <v>9</v>
+      </c>
+      <c r="E39">
+        <v>100</v>
+      </c>
+      <c r="F39" t="s">
+        <v>10</v>
+      </c>
+      <c r="G39">
+        <v>311.91000000000003</v>
+      </c>
+      <c r="H39" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40">
+        <v>34</v>
+      </c>
+      <c r="C40">
+        <v>1012</v>
+      </c>
+      <c r="D40" t="s">
+        <v>9</v>
+      </c>
+      <c r="E40">
+        <v>100</v>
+      </c>
+      <c r="F40" t="s">
+        <v>10</v>
+      </c>
+      <c r="G40">
+        <v>312.41000000000003</v>
+      </c>
+      <c r="H40" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41">
+        <v>35</v>
+      </c>
+      <c r="C41">
+        <v>1013</v>
+      </c>
+      <c r="D41" t="s">
+        <v>9</v>
+      </c>
+      <c r="E41">
+        <v>100</v>
+      </c>
+      <c r="F41" t="s">
+        <v>10</v>
+      </c>
+      <c r="G41">
+        <v>312.91000000000003</v>
+      </c>
+      <c r="H41" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>13</v>
+      </c>
+      <c r="B42">
+        <v>36</v>
+      </c>
+      <c r="C42">
+        <v>1014</v>
+      </c>
+      <c r="D42" t="s">
+        <v>9</v>
+      </c>
+      <c r="E42">
+        <v>100</v>
+      </c>
+      <c r="F42" t="s">
+        <v>10</v>
+      </c>
+      <c r="G42">
+        <v>313.41000000000003</v>
+      </c>
+      <c r="H42" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>13</v>
+      </c>
+      <c r="B43">
+        <v>37</v>
+      </c>
+      <c r="C43">
+        <v>1015</v>
+      </c>
+      <c r="D43" t="s">
+        <v>9</v>
+      </c>
+      <c r="E43">
+        <v>100</v>
+      </c>
+      <c r="F43" t="s">
+        <v>10</v>
+      </c>
+      <c r="G43">
+        <v>313.91000000000003</v>
+      </c>
+      <c r="H43" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>13</v>
+      </c>
+      <c r="B44">
+        <v>38</v>
+      </c>
+      <c r="C44">
+        <v>1016</v>
+      </c>
+      <c r="D44" t="s">
+        <v>9</v>
+      </c>
+      <c r="E44">
+        <v>100</v>
+      </c>
+      <c r="F44" t="s">
+        <v>10</v>
+      </c>
+      <c r="G44">
+        <v>314.41000000000003</v>
+      </c>
+      <c r="H44" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45">
+        <v>39</v>
+      </c>
+      <c r="C45">
+        <v>1017</v>
+      </c>
+      <c r="D45" t="s">
+        <v>9</v>
+      </c>
+      <c r="E45">
+        <v>100</v>
+      </c>
+      <c r="F45" t="s">
+        <v>10</v>
+      </c>
+      <c r="G45">
+        <v>314.91000000000003</v>
+      </c>
+      <c r="H45" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>13</v>
+      </c>
+      <c r="B46">
+        <v>40</v>
+      </c>
+      <c r="C46">
+        <v>1018</v>
+      </c>
+      <c r="D46" t="s">
+        <v>9</v>
+      </c>
+      <c r="E46">
+        <v>100</v>
+      </c>
+      <c r="F46" t="s">
+        <v>10</v>
+      </c>
+      <c r="G46">
+        <v>315.41000000000003</v>
+      </c>
+      <c r="H46" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47">
+        <v>41</v>
+      </c>
+      <c r="C47">
+        <v>1019</v>
+      </c>
+      <c r="D47" t="s">
+        <v>9</v>
+      </c>
+      <c r="E47">
+        <v>100</v>
+      </c>
+      <c r="F47" t="s">
+        <v>10</v>
+      </c>
+      <c r="G47">
+        <v>315.91000000000003</v>
+      </c>
+      <c r="H47" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>13</v>
+      </c>
+      <c r="B48">
+        <v>42</v>
+      </c>
+      <c r="C48">
+        <v>1020</v>
+      </c>
+      <c r="D48" t="s">
+        <v>9</v>
+      </c>
+      <c r="E48">
+        <v>100</v>
+      </c>
+      <c r="F48" t="s">
+        <v>10</v>
+      </c>
+      <c r="G48">
+        <v>316.41000000000003</v>
+      </c>
+      <c r="H48" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>13</v>
+      </c>
+      <c r="B49">
+        <v>43</v>
+      </c>
+      <c r="C49">
+        <v>1021</v>
+      </c>
+      <c r="D49" t="s">
+        <v>9</v>
+      </c>
+      <c r="E49">
+        <v>100</v>
+      </c>
+      <c r="F49" t="s">
+        <v>10</v>
+      </c>
+      <c r="G49">
+        <v>316.91000000000003</v>
+      </c>
+      <c r="H49" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>13</v>
+      </c>
+      <c r="B50">
+        <v>44</v>
+      </c>
+      <c r="C50">
+        <v>1022</v>
+      </c>
+      <c r="D50" t="s">
+        <v>9</v>
+      </c>
+      <c r="E50">
+        <v>100</v>
+      </c>
+      <c r="F50" t="s">
+        <v>10</v>
+      </c>
+      <c r="G50">
+        <v>317.41000000000003</v>
+      </c>
+      <c r="H50" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>8</v>
+      </c>
+      <c r="B52">
+        <v>45</v>
+      </c>
+      <c r="C52">
+        <v>1023</v>
+      </c>
+      <c r="D52" t="s">
+        <v>9</v>
+      </c>
+      <c r="E52">
+        <v>100</v>
+      </c>
+      <c r="F52" t="s">
+        <v>10</v>
+      </c>
+      <c r="G52">
+        <v>319.91000000000003</v>
+      </c>
+      <c r="H52" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>13</v>
+      </c>
+      <c r="B53">
+        <v>46</v>
+      </c>
+      <c r="C53">
+        <v>1023</v>
+      </c>
+      <c r="D53" t="s">
+        <v>9</v>
+      </c>
+      <c r="E53">
+        <v>50</v>
+      </c>
+      <c r="F53" t="s">
+        <v>10</v>
+      </c>
+      <c r="G53">
+        <v>319.91000000000003</v>
+      </c>
+      <c r="H53" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>11</v>
+      </c>
+      <c r="B54">
+        <v>47</v>
+      </c>
+      <c r="C54">
+        <v>1023</v>
+      </c>
+      <c r="D54" t="s">
+        <v>9</v>
+      </c>
+      <c r="E54">
+        <v>50</v>
+      </c>
+      <c r="F54" t="s">
+        <v>10</v>
+      </c>
+      <c r="G54">
+        <v>319.91000000000003</v>
+      </c>
+      <c r="H54" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
HPS support for all ITCH messages
- Tested partial cancel + delete
- Updated gitignore
- Updated M3_demo.py to support vector script
</commit_message>
<xml_diff>
--- a/gen_test_vectors/test_vectors.xlsx
+++ b/gen_test_vectors/test_vectors.xlsx
@@ -1,21 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sofiya\OneDrive\Desktop\ELEC_491_local\hft_top\gen_test_vectors\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61500C75-B2E9-4DE8-995F-C8DD7BBB1B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Exchange_Test"/>
-    <sheet r:id="rId2" sheetId="2" name="NetIO_Test"/>
+    <sheet name="Exchange_Test" sheetId="1" r:id="rId1"/>
+    <sheet name="NetIO_Test" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="13">
   <si>
     <t>Message Type</t>
   </si>
@@ -50,20 +56,19 @@
     <t>AAPL</t>
   </si>
   <si>
-    <t>F</t>
+    <t>X</t>
   </si>
   <si>
     <t>D</t>
-  </si>
-  <si>
-    <t>X</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="7" formatCode="&quot;$&quot;#,##0.00;\-&quot;$&quot;#,##0.00"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -106,35 +111,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="7" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="7" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="7" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="7" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -145,10 +147,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -186,71 +188,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -278,7 +280,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -301,11 +303,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -314,13 +316,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -330,7 +332,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -339,7 +341,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -348,7 +350,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -356,10 +358,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -424,120 +426,117 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="4" width="12.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="7.719285714285714" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>100</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="2">
         <v>280</v>
       </c>
-      <c r="H2" s="1"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
-      <c r="A3" s="1" t="s">
+    </row>
+    <row r="3" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="2">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2">
-        <v>2</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>200</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="2">
         <v>281</v>
       </c>
-      <c r="H3" s="1"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
-      <c r="A4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="2">
+    </row>
+    <row r="4" spans="1:8" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="1">
         <v>3</v>
       </c>
-      <c r="C4" s="2">
-        <v>2</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>200</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="2">
         <v>281</v>
       </c>
-      <c r="H4" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -545,120 +544,140 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="4" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="10.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="10.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="4" width="8.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="4" width="9.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="6" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="4" width="10.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="1">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="1">
         <v>100</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="2">
         <v>280</v>
       </c>
-      <c r="H2" s="1"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="1" t="s">
+    </row>
+    <row r="3" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="1">
+        <v>200</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" s="2">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2">
-        <v>2</v>
-      </c>
-      <c r="C3" s="2">
-        <v>2</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="B4" s="1">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="2">
-        <v>200</v>
-      </c>
-      <c r="F3" s="1" t="s">
+      <c r="E4" s="1">
+        <v>50</v>
+      </c>
+      <c r="F4" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G4" s="2">
         <v>281</v>
       </c>
-      <c r="H3" s="1"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="1" t="s">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="2">
-        <v>3</v>
-      </c>
-      <c r="C4" s="2">
-        <v>2</v>
-      </c>
-      <c r="D4" s="1" t="s">
+      <c r="B5" s="1">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="2">
-        <v>200</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="E5" s="1">
+        <v>150</v>
+      </c>
+      <c r="F5" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G5" s="2">
         <v>281</v>
       </c>
-      <c r="H4" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>